<commit_message>
xlstream-eval: fix text coercion, add unit tests, expand conformance coverage
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/issues/issue-140-aggregate-literal-args.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/issues/issue-140-aggregate-literal-args.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10510"/>
-  <workbookPr defaultThemeVersion="124226"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jason/Projects/xlstream-fix-sum-literal-args/crates/xlstream-eval/tests/fixtures/issues/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_68BE049332E62ED6EFFC9890E25EF2319714FB65" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFC3E33F-DC34-3F4F-A791-7A37908F6105}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="500" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -91,9 +92,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -131,7 +132,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -165,7 +166,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -200,10 +200,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -377,7 +376,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -393,50 +392,44 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A3">
+        <f>SUM(TRUE,1,FALSE)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4">
+        <f>SUM(42)</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5">
         <f>AVERAGE(1,2,3)</f>
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6">
+        <f>AVERAGE(42)</f>
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7">
+        <f>COUNT(1,2,3)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8">
+        <f>COUNTA(1,2,TRUE)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10">
         <f>MAX(1,2,3)</f>
         <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5">
-        <f>MIN(1,2,3)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6">
-        <f>SUM(TRUE,1,FALSE)</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <f>MEDIAN(1,5,3)</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <f>SUM(42)</f>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9">
-        <f>AVERAGE(42)</f>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10">
-        <f>MIN(-5,0,5)</f>
-        <v>-5</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
@@ -445,7 +438,49 @@
         <v>5</v>
       </c>
     </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12">
+        <f>MIN(1,2,3)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <f>MIN(-5,0,5)</f>
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <f>MEDIAN(1,5,3)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <f>PRODUCT(2,3,4)</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <f>PRODUCT(TRUE,5)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <f>SUM("5",1)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="e">
+        <f>SUM(1,1/0)</f>
+        <v>#DIV/0!</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>